<commit_message>
WorldBox tests: add session 2 (underdog win), split stats by session, 2/2 win rate
</commit_message>
<xml_diff>
--- a/training/experiments/worldbox_session_2026-10-11.xlsx
+++ b/training/experiments/worldbox_session_2026-10-11.xlsx
@@ -7,9 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Population Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 Population" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 Strategy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Population" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Strategy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Stats" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,6 +430,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Faction played</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Starting position</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Final score (mine vs top rival)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Main winning move</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sobo (Mamydet Realm)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Largest of 4 (9 pop)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>24 vs 16 (village pop)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Far-side settler spawning + lightning on rival</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Kamiwood (Saba Imperium)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Underdog: 58 vs 99 (kingdom pop)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>119 vs 102 (kingdom pop)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Far-side settler spawning (5 waves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Win rate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2/2 (100%)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -615,7 +763,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -911,7 +1059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1091,4 +1239,758 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>WorldBox - God Simulator (EasyFun cloud), same world as S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Claude (Chrome side panel) for Gavin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Faction</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kamiwood village / Saba Imperium kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Underdog: beat the S1 winner (Mamydet Realm) from behind</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WIN (largest kingdom at session end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Win condition used</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Highest kingdom population when session ended</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Starting Kamiwood village pop</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Starting kingdom pops</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Saba Imperium 58 vs Mamydet Realm 99</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Final Saba Imperium pop</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Final Mamydet Realm pop</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Final Kamiwood village pop</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lightning strikes used (approx.)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Humans spawned (approx.)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rain used</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Between-session event</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mamydet Realm won a War of Conquest (Good Clash of Mamydet Realm), likely absorbing Grenlbourg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Notable event</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Old Mamydet king died; King Vurtelle crowned during S2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Checkpoint</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kamiwood (village)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sobo (village)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Saba Imperium (kingdom)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Mamydet Realm (kingdom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Session start</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Settler wave 1 (west side)</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>35</v>
+      </c>
+      <c r="D3" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lightning on Sobo, forest fire</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>38 (shown as Wulorah)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>After wave 2</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>49</v>
+      </c>
+      <c r="E5" t="n">
+        <v>58</v>
+      </c>
+      <c r="F5" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lightning on Mamydet villages</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>56</v>
+      </c>
+      <c r="F6" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wave 3</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Waves 4-5 (40 settlers)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>102</v>
+      </c>
+      <c r="F8" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>102</v>
+      </c>
+      <c r="E9" t="n">
+        <v>119</v>
+      </c>
+      <c r="F9" t="n">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Chose underdog Kamiwood</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Test the S1 playbook from behind</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Same strategy, harder start</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Settlers spawned on the far (west) side</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>20 -&gt; 35 -&gt; 49</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The far-side trick works reliably</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lightning on Sobo capital</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Big forest fire; village 57 -&gt; 38</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fire hits buildings and trees more than people</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lightning across Mamydet villages</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>99 -&gt; 95 only</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Disasters are weak against a big spread-out kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rain on a stray fire near Kamiwood</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Protected home village</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Defend your own forests</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Two 20-settler waves</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Kamiwood 76 -&gt; 102; kingdom 119</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Volume of spawns decides the outcome</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sapient population (world)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>151</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Start of S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total playtime</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0:27:05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Trees grown</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1069</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Flora grown</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2647</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pixels exploded</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>85</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Creatures created</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>387</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Creatures born</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>145</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total creatures died</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>306</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Subspecies created</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>167</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Subspecies extinct</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>114</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
WorldBox tests: add session 3 (conquest win via held-press exploit), 3/3 win rate [from side-panel Claude as Pocket Sophia]
</commit_message>
<xml_diff>
--- a/training/experiments/worldbox_session_2026-10-11.xlsx
+++ b/training/experiments/worldbox_session_2026-10-11.xlsx
@@ -14,7 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Population" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2 Strategy" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Stats" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3 Summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S3 Strategy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="World Stats" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -549,16 +551,250 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mamydet Realm (Sobo)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Behind: 102 vs 119 (kingdom pop)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WIN (conquest)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>292 vs 0 (Saba Imperium conquered)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Held-press exploit: sink + flood rival capital, then war</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Win rate</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3/3 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>S3 rules changed mid-session from magnet-only to the combined plan (Gavin asked for a creative solution combining all three ideas).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sapient population (world)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>151</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Start of S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total playtime</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0:27:05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Trees grown</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1069</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Win rate</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2/2 (100%)</t>
+          <t>Flora grown</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2647</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pixels exploded</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>85</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Creatures created</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>387</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Creatures born</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>145</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total creatures died</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>306</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Subspecies created</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>167</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>During S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Subspecies extinct</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>114</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>During S2</t>
         </is>
       </c>
     </row>
@@ -1813,180 +2049,444 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stat</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>When</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sapient population (world)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>151</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Start of S2</t>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total playtime</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0:27:05</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Pocket Sophia (Claude in the Chrome side panel, using SOPHIA.md style)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trees grown</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1069</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Faction</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mamydet Realm (capital Sobo)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Flora grown</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2647</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Starting kingdom pops</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mamydet Realm 102 vs Saba Imperium 119</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pixels exploded</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>85</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Planned category</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Magnet-only (no spawning, no lightning)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Creatures created</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>387</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Actual category</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Combined: sink + flood + magnet + soil (rules changed at Gavin's request)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Creatures born</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>145</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>During S2</t>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WIN by conquest: Saba Imperium reduced to 0 in War of Conquest</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Total creatures died</t>
+          <t>Final Mamydet Realm pop</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>306</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>During S2</t>
-        </is>
+        <v>292</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Subspecies created</t>
+          <t>Final Sobo village pop</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>167</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>During S2</t>
-        </is>
+        <v>148</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Subspecies extinct</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>114</v>
+          <t>War</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Clash of Broken Bones (War of Conquest), Mamydet attacker; defender losses 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Saba king deaths</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Demicha died when his capital was sunk; Gillin crowned</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Settlers spawned</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lightning strikes</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Key exploit</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Held-press: scripted slow pointer events let held tools work through the cloud stream</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Read training/research/game_exploits.md</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Picked magnet + water combo; set magnet-only category</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Know your category up front</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Magnet via instant drag / tap</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Failed: Kamiwood 136 -&gt; 138</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Obstacle: held-drag. Instant input cannot hold a tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Magnet at night</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Few targets</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Edge: at night units are indoors</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Terrain, TNT, grenade via taps</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>All failed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Same obstacle: they are held/paint tools</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lightning tap test</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Worked</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Isolate the variable before blaming the tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Held-press exploit (scripted pointer down/move/up)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Held tools work</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Change the method, not the effort</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Deep Ocean pit over Kamiwood center</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Capital sunk; King Demicha died</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Win condition is people, so take their land</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rain over the pit</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pit flooded into a bay</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tools combine: pit + rain = sea</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Magnet (held) into bay</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Kamiwood 140 -&gt; 132</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Works, but night limits it</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Forest Soil on Mamydet land</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>During S2</t>
+          <t>Bare soil; biome seeds not found</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dead end: needs seeds; did not hurt growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Waited</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mamydet declared war and conquered Saba (292 vs 0)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A weakened rival invites the AI to finish the job</t>
         </is>
       </c>
     </row>

</xml_diff>